<commit_message>
Added support for 2.5 week courses in coursepackages to be read together.
</commit_message>
<xml_diff>
--- a/backend/scripts/EducationData.xlsx
+++ b/backend/scripts/EducationData.xlsx
@@ -5,11 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Kurser" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Kurspaket" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Kurser" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Kurspaket" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="220">
   <si>
     <t xml:space="preserve">Program</t>
   </si>
@@ -681,9 +681,6 @@
   </si>
   <si>
     <t xml:space="preserve">VOXACE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anatomi och fysiologi Nvå 1a2</t>
   </si>
 </sst>
 </file>
@@ -694,10 +691,10 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
@@ -720,14 +717,14 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -735,7 +732,14 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
@@ -750,19 +754,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.4999"/>
+        <fgColor rgb="FF4E95D9"/>
         <bgColor rgb="FF3366FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2"/>
+        <fgColor rgb="FFE8E8E8"/>
         <bgColor rgb="FFDCEAF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.8999"/>
+        <fgColor rgb="FFDCEAF7"/>
         <bgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
@@ -801,7 +805,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -831,6 +835,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -914,185 +922,13 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office-tema">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0e2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="e8e8e8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="e97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196b24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="a02b93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4ea72e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607d"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E84"/>
-  <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7578125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="43.33"/>
@@ -2192,11 +2028,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C80" s="8" t="s">
         <v>161</v>
       </c>
       <c r="D80" s="4" t="n">
@@ -2248,14 +2084,14 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B84" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C84" s="1" t="s">
+      <c r="C84" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="E84" s="1" t="n">
+      <c r="E84" s="8" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2276,7 +2112,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F143"/>
-  <sheetFormatPr defaultColWidth="8.75390625" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7578125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="49.89"/>
@@ -2313,16 +2149,16 @@
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5"/>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="9" t="n">
         <v>900</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <v>45</v>
       </c>
     </row>
@@ -2469,16 +2305,16 @@
       <c r="E13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -2553,16 +2389,16 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
+      <c r="B21" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2623,16 +2459,16 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2693,16 +2529,16 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="D33" s="8" t="n">
+      <c r="D33" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E33" s="8" t="n">
+      <c r="E33" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2763,16 +2599,16 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="D39" s="8" t="n">
+      <c r="D39" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E39" s="8" t="n">
+      <c r="E39" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -2833,16 +2669,16 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="D45" s="8" t="n">
+      <c r="D45" s="9" t="n">
         <v>900</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="E45" s="9" t="n">
         <v>45</v>
       </c>
     </row>
@@ -2973,16 +2809,16 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="8" t="s">
+      <c r="B56" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C56" s="8" t="s">
+      <c r="C56" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="D56" s="8" t="n">
+      <c r="D56" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="E56" s="8" t="n">
+      <c r="E56" s="9" t="n">
         <v>25</v>
       </c>
     </row>
@@ -3057,16 +2893,16 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B63" s="8" t="s">
+      <c r="B63" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="C63" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="D63" s="8" t="n">
+      <c r="D63" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E63" s="8" t="n">
+      <c r="E63" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3127,16 +2963,16 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B69" s="8" t="s">
+      <c r="B69" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C69" s="8" t="s">
+      <c r="C69" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="D69" s="8" t="n">
+      <c r="D69" s="9" t="n">
         <v>400</v>
       </c>
-      <c r="E69" s="8" t="n">
+      <c r="E69" s="9" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3202,16 +3038,16 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="C75" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="D75" s="8" t="n">
+      <c r="D75" s="9" t="n">
         <v>1400</v>
       </c>
-      <c r="E75" s="8" t="n">
+      <c r="E75" s="9" t="n">
         <v>70</v>
       </c>
     </row>
@@ -3398,16 +3234,16 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B90" s="8" t="s">
+      <c r="B90" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C90" s="8" t="s">
+      <c r="C90" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="D90" s="8" t="n">
+      <c r="D90" s="9" t="n">
         <v>1400</v>
       </c>
-      <c r="E90" s="8" t="n">
+      <c r="E90" s="9" t="n">
         <v>70</v>
       </c>
     </row>
@@ -3599,16 +3435,16 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B106" s="8" t="s">
+      <c r="B106" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="C106" s="8" t="s">
+      <c r="C106" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="D106" s="8" t="n">
+      <c r="D106" s="9" t="n">
         <v>1500</v>
       </c>
-      <c r="E106" s="8" t="n">
+      <c r="E106" s="9" t="n">
         <v>75</v>
       </c>
     </row>
@@ -3655,34 +3491,36 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B110" s="9" t="s">
+      <c r="B110" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C110" s="9" t="s">
+      <c r="C110" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D110" s="9" t="n">
+      <c r="D110" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E110" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F110" s="9" t="s">
+      <c r="E110" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F110" s="10" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B111" s="9" t="s">
+      <c r="B111" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="C111" s="9" t="s">
+      <c r="C111" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="D111" s="9" t="n">
+      <c r="D111" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E111" s="9"/>
-      <c r="F111" s="9"/>
+      <c r="E111" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F111" s="10"/>
     </row>
     <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B112" s="1" t="s">
@@ -3895,34 +3733,36 @@
       </c>
     </row>
     <row r="128" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B128" s="9" t="s">
+      <c r="B128" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C128" s="9" t="s">
+      <c r="C128" s="10" t="s">
         <v>217</v>
       </c>
-      <c r="D128" s="9" t="n">
+      <c r="D128" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E128" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F128" s="9" t="s">
+      <c r="E128" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F128" s="10" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B129" s="9" t="s">
+      <c r="B129" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="C129" s="9" t="s">
+      <c r="C129" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D129" s="9" t="n">
+      <c r="D129" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E129" s="9"/>
-      <c r="F129" s="9"/>
+      <c r="E129" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F129" s="10"/>
     </row>
     <row r="130" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B130" s="1" t="s">
@@ -4037,34 +3877,36 @@
       </c>
     </row>
     <row r="139" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B139" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="C139" s="9" t="s">
+      <c r="B139" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C139" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D139" s="9" t="n">
+      <c r="D139" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E139" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="F139" s="9" t="s">
+      <c r="E139" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F139" s="10" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B140" s="9" t="s">
+      <c r="B140" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="C140" s="9" t="s">
+      <c r="C140" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="D140" s="9" t="n">
+      <c r="D140" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="E140" s="9"/>
-      <c r="F140" s="9"/>
+      <c r="E140" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B141" s="1" t="s">

</xml_diff>